<commit_message>
feat(demo): generate the showcase workbook and give it a chart
showcase.xlsx was a committed binary with no generator, so nothing kept it
honest. It is now produced by scripts/create-demo-workbook.ts in the same
shape as the deck and doc generators, with a pinned zip date so the output is
byte-stable, and CI regenerates it and diffs against the committed file.

The Dashboard sheet gains a column chart of revenue by region, anchored beside
the table. Its category and value caches are built from the same rows the
cells are written from, so the cache cannot disagree with the sheet it
references.

Regenerating the workbook changes the collaboration seed derived from it, so
xlsx.bin is rebuilt to match; the docx and pptx seeds are untouched. The
generator also emits the true mergeCells count, which the original declared
as 2 while carrying three children.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/demo/public/showcase.xlsx
+++ b/apps/demo/public/showcase.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="54">
   <si>
     <t xml:space="preserve">Q3 Sales Dashboard</t>
   </si>
@@ -64,13 +64,34 @@
     <t xml:space="preserve">Result</t>
   </si>
   <si>
+    <t xml:space="preserve">Values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
     <t xml:space="preserve">SUM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alpha</t>
   </si>
   <si>
     <t xml:space="preserve">AVERAGE</t>
   </si>
   <si>
+    <t xml:space="preserve">Beta</t>
+  </si>
+  <si>
     <t xml:space="preserve">MIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gamma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northeast</t>
   </si>
   <si>
     <t xml:space="preserve">MAX</t>
@@ -98,27 +119,6 @@
   </si>
   <si>
     <t xml:space="preserve">End of month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alpha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gamma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Northeast</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -276,6 +276,182 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
+              <a:t>Revenue by region</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472C4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$5:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$C$5:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>386400</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>274850</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>512300</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>331200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:axId val="553771648"/>
+        <c:axId val="553773184"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="553771648"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="553773184"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="553773184"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="&quot;$&quot;#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="553771648"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Revenue by region"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F11"/>
@@ -424,11 +600,12 @@
       <c r="F11" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>
   </mergeCells>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -456,13 +633,13 @@
         <v>16</v>
       </c>
       <c r="E2" t="s" s="3">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s" s="3">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s" s="3">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="K2" t="s" s="3">
         <v>2</v>
@@ -470,7 +647,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="11">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <f>SUM(E3:E7)</f>
@@ -479,7 +656,7 @@
         <v>12</v>
       </c>
       <c r="H3" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="I3">
         <v>100</v>
@@ -490,7 +667,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="11">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <f>AVERAGE(E3:E7)</f>
@@ -499,7 +676,7 @@
         <v>47</v>
       </c>
       <c r="H4" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="I4">
         <v>200</v>
@@ -510,7 +687,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="11">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <f>MIN(E3:E7)</f>
@@ -519,18 +696,18 @@
         <v>8</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="I5">
         <v>300</v>
       </c>
       <c r="K5" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="11">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B6">
         <f>MAX(E3:E7)</f>
@@ -544,7 +721,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="11">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B7">
         <f>IF(B3&gt;100,"Over budget","Within budget")</f>
@@ -555,7 +732,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="11">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="B8">
         <f>IFS(B4&gt;=40,"High",B4&gt;=20,"Medium",TRUE,"Low")</f>
@@ -563,7 +740,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="11">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B9">
         <f>VLOOKUP("Gamma",H3:I5,2,FALSE)</f>
@@ -571,7 +748,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="11">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <f>COUNTIF(K3:K6,"North*")</f>
@@ -579,7 +756,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="11">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B11" s="6">
         <f>B4/B6</f>
@@ -587,7 +764,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="11">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B12">
         <f>TEXT(B4,"#,##0.00")</f>
@@ -595,7 +772,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="11">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B13" s="5">
         <f>TODAY()</f>
@@ -603,7 +780,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="11">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B14" s="5">
         <f>EOMONTH(TODAY(),0)</f>

</xml_diff>